<commit_message>
docs(waterfall): ejemplos ficticios actualizados (proyección parcial, fechas distintas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWmFk3cyaXSqjsmvoCZymx
</commit_message>
<xml_diff>
--- a/docs/waterfall/waterfall-2026-2027-allpa-peru-proporcional-ficticio.xlsx
+++ b/docs/waterfall/waterfall-2026-2027-allpa-peru-proporcional-ficticio.xlsx
@@ -903,7 +903,7 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>Saldo Final Caja (USD) = saldo inicial + flujo proyectado</t>
+          <t>Proyección parcial (USD): mes del corte pendiente de conciliar</t>
         </is>
       </c>
       <c r="B20" s="10">
@@ -946,7 +946,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>Informativo — fuera de la identidad, no suma</t>
+          <t>Fuera de la proyección parcial — no suma</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
@@ -998,168 +998,140 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>Saldo final × % de propiedad (atribuible; no es caja consolidada)</t>
+          <t>Flujo del mes del corte EXCLUIDO, pendiente de conciliar (ver fecha del saldo de cada sociedad)</t>
         </is>
       </c>
       <c r="B22" s="10">
-        <v>-966268</v>
+        <v>-3283.5</v>
       </c>
       <c r="C22" s="10">
-        <v>-407202.4</v>
+        <v>-48399.5</v>
       </c>
       <c r="D22" s="10">
-        <v>566351.1</v>
+        <v>-22697</v>
       </c>
       <c r="E22" s="10">
-        <v>-76850</v>
+        <v>-12400</v>
       </c>
       <c r="F22" s="10">
-        <v>3557451</v>
+        <v>-87622</v>
       </c>
       <c r="G22" s="10">
-        <v>-278545</v>
+        <v>-29252</v>
       </c>
       <c r="H22" s="10">
-        <v>-262526.57790216006</v>
+        <v>274979.8918900801</v>
       </c>
       <c r="I22" s="10">
         <f>SUM(B22:H22)</f>
-        <v>2132410.12209784</v>
+        <v>71325.89189008012</v>
       </c>
       <c r="J22" s="10">
-        <v>-319305.44</v>
+        <v>-77044.41</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>Flujo del mes del corte (no incluido: no se puede separar lo ya incorporado al banco)</t>
+          <t>Simulación: si TODO el flujo del mes del corte estuviera pendiente (no es el saldo correcto, ni un mínimo, ni un máximo)</t>
         </is>
       </c>
       <c r="B23" s="10">
-        <v>-3283.5</v>
+        <v>-969551.5</v>
       </c>
       <c r="C23" s="10">
-        <v>-48399.5</v>
+        <v>-557402.5</v>
       </c>
       <c r="D23" s="10">
-        <v>-22697</v>
+        <v>606582</v>
       </c>
       <c r="E23" s="10">
-        <v>-12400</v>
+        <v>-89250</v>
       </c>
       <c r="F23" s="10">
-        <v>-87622</v>
+        <v>3469829</v>
       </c>
       <c r="G23" s="10">
-        <v>-29252</v>
+        <v>-307797</v>
       </c>
       <c r="H23" s="10">
-        <v>274979.8918900801</v>
+        <v>12453.31398792006</v>
       </c>
       <c r="I23" s="10">
         <f>SUM(B23:H23)</f>
-        <v>71325.89189008012</v>
+        <v>2164863.31398792</v>
       </c>
       <c r="J23" s="10">
-        <v>-77044.41</v>
+        <v>-715655.29</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>Saldo final si el mes del corte estuviera completo pendiente</t>
+          <t>Flujo ya transcurrido de la temporada (histórico, ya en el saldo bancario)</t>
         </is>
       </c>
       <c r="B24" s="10">
-        <v>-969551.5</v>
+        <v>-9850.5</v>
       </c>
       <c r="C24" s="10">
-        <v>-557402.5</v>
+        <v>-153807.5</v>
       </c>
       <c r="D24" s="10">
-        <v>606582</v>
+        <v>-92703</v>
       </c>
       <c r="E24" s="10">
-        <v>-89250</v>
+        <v>-37050</v>
       </c>
       <c r="F24" s="10">
-        <v>3469829</v>
+        <v>-254920</v>
       </c>
       <c r="G24" s="10">
-        <v>-307797</v>
+        <v>-64138</v>
       </c>
       <c r="H24" s="10">
-        <v>12453.31398792006</v>
+        <v>351955.4143533999</v>
       </c>
       <c r="I24" s="10">
         <f>SUM(B24:H24)</f>
-        <v>2164863.31398792</v>
+        <v>-260513.5856466001</v>
       </c>
       <c r="J24" s="10">
-        <v>-715655.29</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" t="inlineStr" s="0">
-        <is>
-          <t>Flujo ya transcurrido de la temporada (histórico, ya en el saldo bancario)</t>
-        </is>
-      </c>
-      <c r="B25" s="10">
-        <v>-9850.5</v>
-      </c>
-      <c r="C25" s="10">
-        <v>-153807.5</v>
-      </c>
-      <c r="D25" s="10">
-        <v>-92703</v>
-      </c>
-      <c r="E25" s="10">
-        <v>-37050</v>
-      </c>
-      <c r="F25" s="10">
-        <v>-254920</v>
-      </c>
-      <c r="G25" s="10">
-        <v>-64138</v>
-      </c>
-      <c r="H25" s="10">
-        <v>351955.4143533999</v>
-      </c>
-      <c r="I25" s="10">
-        <f>SUM(B25:H25)</f>
-        <v>-260513.5856466001</v>
-      </c>
-      <c r="J25" s="10">
         <v>-167127.79000000004</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr" s="6">
+        <is>
+          <t>VISTA GERENCIAL DE CAJA, no consolidación contable: suma las 6 sociedades al 100% y Allpa Farms Perú al 26% de su caja. Bajo IAS 28 una JV se registra por método de participación y su caja no se suma. Allpa Farms: JV por método de participación, se muestran aparte al 100% y NO suman al total.</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="6">
         <is>
-          <t>VISTA GERENCIAL DE CAJA, no consolidación contable: suma las 6 sociedades al 100% y Allpa Farms Perú al 26% de su caja. Bajo IAS 28 una JV se registra por método de participación y su caja no se suma. Allpa Farms: JV por método de participación, se muestran aparte al 100% y NO suman al total.</t>
+          <t>Saldo de caja INCOMPLETO: se excluyen cuentas sin TC guardado de Frisku Foods.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="6">
         <is>
-          <t>Saldo de caja INCOMPLETO: se excluyen cuentas sin TC guardado de Frisku Foods.</t>
+          <t>El total suma saldos bancarios a 6 fechas distintas (15-09-2026 a 12-10-2026): no es la caja del grupo a una fecha común.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="6">
         <is>
-          <t>Saldo inicial + flujo proyectado = saldo final. El mes del corte no entra (la proyección es mensual y no separa lo ya incorporado al banco); se informa aparte. Los meses anteriores al corte son históricos y no suman.</t>
+          <t>PROYECCIÓN PARCIAL, no saldo final definitivo: saldo al corte + flujo de los meses posteriores al mes del corte. El flujo del mes del corte está EXCLUIDO y pendiente de conciliar (ni completo ni cero). La fila de simulación no es el saldo correcto, ni un mínimo, ni un máximo. Los meses anteriores al corte son históricos y no suman.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="6">
         <is>
-          <t>Las subsidiarias van al 100% de su caja; la fila «atribuible» (saldo final × % de propiedad) es informativa y no es caja consolidada.</t>
+          <t>Las subsidiarias van al 100% de su caja; la inclusión proporcional de JV es una vista gerencial, no IAS 28.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1287,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D5" s="10">
@@ -1675,7 +1647,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D17" s="10">
@@ -2035,7 +2007,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D29" s="10">
@@ -2395,7 +2367,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D41" s="10">
@@ -2755,7 +2727,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D53" s="10">
@@ -3087,7 +3059,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D64" s="10">
@@ -3478,7 +3450,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Mes del corte (no incluido)</t>
+          <t>Mes del corte (excluido, pendiente de conciliar)</t>
         </is>
       </c>
       <c r="D77" s="10">

</xml_diff>